<commit_message>
Use whole-dollar unit and line prices that sum to 5860.
Keep the first and third items unchanged, leave quantities as-is, and keep 22% VAT totaling 7149.20.

Co-authored-by: alexanderp-cell <alexanderp-cell@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/11111.xlsx
+++ b/11111.xlsx
@@ -516,22 +516,22 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="3" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="2" fontId="3" fillId="3" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="3" fillId="3" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="3" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="3" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="3" fillId="3" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="3" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="3" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="3" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1075,7 +1075,7 @@
       <c r="K3" s="15" t="n">
         <v>0.22</v>
       </c>
-      <c r="L3" s="55" t="n">
+      <c r="L3" s="54" t="n">
         <v>12.2</v>
       </c>
     </row>
@@ -1112,17 +1112,17 @@
           <t>ea</t>
         </is>
       </c>
-      <c r="I4" s="56" t="n">
-        <v>55.73</v>
-      </c>
-      <c r="J4" s="55" t="n">
-        <v>55.73</v>
+      <c r="I4" s="55" t="n">
+        <v>56</v>
+      </c>
+      <c r="J4" s="56" t="n">
+        <v>56</v>
       </c>
       <c r="K4" s="15" t="n">
         <v>0.22</v>
       </c>
-      <c r="L4" s="55" t="n">
-        <v>67.98999999999999</v>
+      <c r="L4" s="54" t="n">
+        <v>68.31999999999999</v>
       </c>
     </row>
     <row r="5" ht="14.65" customHeight="1" thickBot="1">
@@ -1167,7 +1167,7 @@
       <c r="K5" s="15" t="n">
         <v>0.22</v>
       </c>
-      <c r="L5" s="55" t="n">
+      <c r="L5" s="54" t="n">
         <v>12.2</v>
       </c>
     </row>
@@ -1204,17 +1204,17 @@
           <t>ea</t>
         </is>
       </c>
-      <c r="I6" s="56" t="n">
-        <v>111.45</v>
-      </c>
-      <c r="J6" s="55" t="n">
-        <v>111.45</v>
+      <c r="I6" s="55" t="n">
+        <v>111</v>
+      </c>
+      <c r="J6" s="56" t="n">
+        <v>111</v>
       </c>
       <c r="K6" s="15" t="n">
         <v>0.22</v>
       </c>
-      <c r="L6" s="55" t="n">
-        <v>135.97</v>
+      <c r="L6" s="54" t="n">
+        <v>135.42</v>
       </c>
     </row>
     <row r="7" ht="14.65" customHeight="1" thickBot="1">
@@ -1250,17 +1250,17 @@
           <t>ea</t>
         </is>
       </c>
-      <c r="I7" s="56" t="n">
-        <v>55.73</v>
-      </c>
-      <c r="J7" s="55" t="n">
-        <v>278.65</v>
+      <c r="I7" s="55" t="n">
+        <v>56</v>
+      </c>
+      <c r="J7" s="56" t="n">
+        <v>280</v>
       </c>
       <c r="K7" s="15" t="n">
         <v>0.22</v>
       </c>
-      <c r="L7" s="55" t="n">
-        <v>339.95</v>
+      <c r="L7" s="54" t="n">
+        <v>341.6</v>
       </c>
     </row>
     <row r="8" ht="14.65" customHeight="1" thickBot="1">
@@ -1296,17 +1296,17 @@
           <t>ea</t>
         </is>
       </c>
-      <c r="I8" s="56" t="n">
-        <v>55.73</v>
-      </c>
-      <c r="J8" s="55" t="n">
-        <v>55.73</v>
+      <c r="I8" s="55" t="n">
+        <v>56</v>
+      </c>
+      <c r="J8" s="56" t="n">
+        <v>56</v>
       </c>
       <c r="K8" s="15" t="n">
         <v>0.22</v>
       </c>
-      <c r="L8" s="55" t="n">
-        <v>67.98999999999999</v>
+      <c r="L8" s="54" t="n">
+        <v>68.31999999999999</v>
       </c>
     </row>
     <row r="9" ht="14.65" customHeight="1" thickBot="1">
@@ -1342,17 +1342,17 @@
           <t>ea</t>
         </is>
       </c>
-      <c r="I9" s="56" t="n">
-        <v>167.18</v>
-      </c>
-      <c r="J9" s="55" t="n">
-        <v>167.18</v>
+      <c r="I9" s="55" t="n">
+        <v>167</v>
+      </c>
+      <c r="J9" s="56" t="n">
+        <v>167</v>
       </c>
       <c r="K9" s="15" t="n">
         <v>0.22</v>
       </c>
-      <c r="L9" s="55" t="n">
-        <v>203.96</v>
+      <c r="L9" s="54" t="n">
+        <v>203.74</v>
       </c>
     </row>
     <row r="10" ht="14.65" customHeight="1" thickBot="1">
@@ -1388,17 +1388,17 @@
           <t>ea</t>
         </is>
       </c>
-      <c r="I10" s="56" t="n">
-        <v>1582.6</v>
-      </c>
-      <c r="J10" s="55" t="n">
-        <v>1582.6</v>
+      <c r="I10" s="55" t="n">
+        <v>1583</v>
+      </c>
+      <c r="J10" s="56" t="n">
+        <v>1583</v>
       </c>
       <c r="K10" s="15" t="n">
         <v>0.22</v>
       </c>
-      <c r="L10" s="55" t="n">
-        <v>1930.77</v>
+      <c r="L10" s="54" t="n">
+        <v>1931.26</v>
       </c>
     </row>
     <row r="11" ht="14.65" customHeight="1" thickBot="1">
@@ -1434,17 +1434,17 @@
           <t>ea</t>
         </is>
       </c>
-      <c r="I11" s="56" t="n">
-        <v>334.35</v>
-      </c>
-      <c r="J11" s="55" t="n">
-        <v>334.35</v>
+      <c r="I11" s="55" t="n">
+        <v>334</v>
+      </c>
+      <c r="J11" s="56" t="n">
+        <v>334</v>
       </c>
       <c r="K11" s="15" t="n">
         <v>0.22</v>
       </c>
-      <c r="L11" s="55" t="n">
-        <v>407.91</v>
+      <c r="L11" s="54" t="n">
+        <v>407.48</v>
       </c>
     </row>
     <row r="12" ht="14.65" customHeight="1" thickBot="1">
@@ -1480,17 +1480,17 @@
           <t>ea</t>
         </is>
       </c>
-      <c r="I12" s="56" t="n">
-        <v>111.45</v>
-      </c>
-      <c r="J12" s="55" t="n">
-        <v>111.45</v>
+      <c r="I12" s="55" t="n">
+        <v>111</v>
+      </c>
+      <c r="J12" s="56" t="n">
+        <v>111</v>
       </c>
       <c r="K12" s="15" t="n">
         <v>0.22</v>
       </c>
-      <c r="L12" s="55" t="n">
-        <v>135.97</v>
+      <c r="L12" s="54" t="n">
+        <v>135.42</v>
       </c>
     </row>
     <row r="13" ht="14.65" customHeight="1" thickBot="1">
@@ -1526,17 +1526,17 @@
           <t>ea</t>
         </is>
       </c>
-      <c r="I13" s="56" t="n">
-        <v>55.73</v>
-      </c>
-      <c r="J13" s="55" t="n">
-        <v>55.73</v>
+      <c r="I13" s="55" t="n">
+        <v>56</v>
+      </c>
+      <c r="J13" s="56" t="n">
+        <v>56</v>
       </c>
       <c r="K13" s="15" t="n">
         <v>0.22</v>
       </c>
-      <c r="L13" s="55" t="n">
-        <v>67.98999999999999</v>
+      <c r="L13" s="54" t="n">
+        <v>68.31999999999999</v>
       </c>
     </row>
     <row r="14" ht="14.65" customHeight="1" thickBot="1">
@@ -1572,17 +1572,17 @@
           <t>ea</t>
         </is>
       </c>
-      <c r="I14" s="56" t="n">
-        <v>39.01</v>
-      </c>
-      <c r="J14" s="55" t="n">
-        <v>78.02</v>
+      <c r="I14" s="55" t="n">
+        <v>78</v>
+      </c>
+      <c r="J14" s="56" t="n">
+        <v>78</v>
       </c>
       <c r="K14" s="15" t="n">
         <v>0.22</v>
       </c>
-      <c r="L14" s="55" t="n">
-        <v>95.18000000000001</v>
+      <c r="L14" s="54" t="n">
+        <v>95.16</v>
       </c>
     </row>
     <row r="15" ht="15.4" customHeight="1" thickBot="1">
@@ -1618,17 +1618,17 @@
           <t>ea</t>
         </is>
       </c>
-      <c r="I15" s="56" t="n">
-        <v>557.25</v>
-      </c>
-      <c r="J15" s="55" t="n">
-        <v>557.25</v>
+      <c r="I15" s="55" t="n">
+        <v>557</v>
+      </c>
+      <c r="J15" s="56" t="n">
+        <v>557</v>
       </c>
       <c r="K15" s="15" t="n">
         <v>0.22</v>
       </c>
-      <c r="L15" s="55" t="n">
-        <v>679.85</v>
+      <c r="L15" s="54" t="n">
+        <v>679.54</v>
       </c>
     </row>
     <row r="16" ht="14.65" customHeight="1" thickBot="1">
@@ -1664,17 +1664,17 @@
           <t>ea</t>
         </is>
       </c>
-      <c r="I16" s="56" t="n">
-        <v>55.73</v>
-      </c>
-      <c r="J16" s="55" t="n">
-        <v>167.18</v>
+      <c r="I16" s="55" t="n">
+        <v>167</v>
+      </c>
+      <c r="J16" s="56" t="n">
+        <v>167</v>
       </c>
       <c r="K16" s="15" t="n">
         <v>0.22</v>
       </c>
-      <c r="L16" s="55" t="n">
-        <v>203.96</v>
+      <c r="L16" s="54" t="n">
+        <v>203.74</v>
       </c>
     </row>
     <row r="17" ht="14.65" customHeight="1" thickBot="1">
@@ -1710,17 +1710,17 @@
           <t>ea</t>
         </is>
       </c>
-      <c r="I17" s="56" t="n">
-        <v>22.29</v>
-      </c>
-      <c r="J17" s="55" t="n">
-        <v>111.45</v>
+      <c r="I17" s="55" t="n">
+        <v>22</v>
+      </c>
+      <c r="J17" s="56" t="n">
+        <v>110</v>
       </c>
       <c r="K17" s="15" t="n">
         <v>0.22</v>
       </c>
-      <c r="L17" s="55" t="n">
-        <v>135.97</v>
+      <c r="L17" s="54" t="n">
+        <v>134.2</v>
       </c>
     </row>
     <row r="18" ht="14.65" customHeight="1" thickBot="1">
@@ -1757,16 +1757,16 @@
         </is>
       </c>
       <c r="I18" s="57" t="n">
-        <v>6.69</v>
-      </c>
-      <c r="J18" s="55" t="n">
-        <v>167.25</v>
+        <v>7</v>
+      </c>
+      <c r="J18" s="56" t="n">
+        <v>175</v>
       </c>
       <c r="K18" s="21" t="n">
         <v>0.22</v>
       </c>
-      <c r="L18" s="55" t="n">
-        <v>204.05</v>
+      <c r="L18" s="54" t="n">
+        <v>213.5</v>
       </c>
     </row>
     <row r="19" ht="15.4" customHeight="1" thickBot="1">
@@ -1803,16 +1803,16 @@
         </is>
       </c>
       <c r="I19" s="58" t="n">
-        <v>1727.4</v>
-      </c>
-      <c r="J19" s="55" t="n">
-        <v>1727.4</v>
+        <v>1713</v>
+      </c>
+      <c r="J19" s="56" t="n">
+        <v>1713</v>
       </c>
       <c r="K19" s="23" t="n">
         <v>0.22</v>
       </c>
-      <c r="L19" s="55" t="n">
-        <v>2107.42</v>
+      <c r="L19" s="54" t="n">
+        <v>2089.86</v>
       </c>
     </row>
     <row r="20" ht="14.65" customHeight="1" thickBot="1">
@@ -1849,16 +1849,16 @@
         </is>
       </c>
       <c r="I20" s="59" t="n">
-        <v>22.29</v>
-      </c>
-      <c r="J20" s="55" t="n">
-        <v>111.45</v>
+        <v>22</v>
+      </c>
+      <c r="J20" s="56" t="n">
+        <v>110</v>
       </c>
       <c r="K20" s="27" t="n">
         <v>0.22</v>
       </c>
-      <c r="L20" s="55" t="n">
-        <v>135.97</v>
+      <c r="L20" s="54" t="n">
+        <v>134.2</v>
       </c>
     </row>
     <row r="21" ht="14.65" customHeight="1" thickBot="1">
@@ -1894,17 +1894,17 @@
           <t>ea</t>
         </is>
       </c>
-      <c r="I21" s="56" t="n">
-        <v>55.73</v>
-      </c>
-      <c r="J21" s="55" t="n">
-        <v>55.73</v>
+      <c r="I21" s="55" t="n">
+        <v>56</v>
+      </c>
+      <c r="J21" s="56" t="n">
+        <v>56</v>
       </c>
       <c r="K21" s="15" t="n">
         <v>0.22</v>
       </c>
-      <c r="L21" s="55" t="n">
-        <v>67.98999999999999</v>
+      <c r="L21" s="54" t="n">
+        <v>68.31999999999999</v>
       </c>
     </row>
     <row r="22" ht="14.65" customHeight="1" thickBot="1">
@@ -1940,17 +1940,17 @@
           <t>ea</t>
         </is>
       </c>
-      <c r="I22" s="56" t="n">
-        <v>5.57</v>
-      </c>
-      <c r="J22" s="55" t="n">
-        <v>111.4</v>
+      <c r="I22" s="55" t="n">
+        <v>6</v>
+      </c>
+      <c r="J22" s="56" t="n">
+        <v>120</v>
       </c>
       <c r="K22" s="15" t="n">
         <v>0.22</v>
       </c>
-      <c r="L22" s="55" t="n">
-        <v>135.91</v>
+      <c r="L22" s="54" t="n">
+        <v>146.4</v>
       </c>
     </row>
     <row r="23">

</xml_diff>